<commit_message>
Retira NFs 3559 e 3560 da conferência de julho (são jun/26)
Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Conferencia_Criteriosa_Lucro_Jul.xlsx
+++ b/Conferencia_Criteriosa_Lucro_Jul.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q54"/>
+  <dimension ref="A1:Q49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,22 +506,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3559</t>
+          <t>3561</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>30/06/2026 15:27:27</t>
+          <t>01/07/2026 13:28:50</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CITOPHARMA MANIPULAÇÃO DE MEDICAMENTOS ESPECIAIS LTDA</t>
+          <t>FRIGOBET FRIGORIFICO INDUSTRIAL BETIM LTDA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>RIBBON CERA ARMOR 110x74 EXTERNO</t>
+          <t>RIBBON CERA 110X450 EXTERNO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -530,31 +530,31 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>297.12</v>
+        <v>525.6</v>
       </c>
       <c r="G2" t="n">
-        <v>167.04</v>
+        <v>360</v>
       </c>
       <c r="H2" t="n">
-        <v>8.913600000000001</v>
+        <v>70</v>
       </c>
       <c r="I2" t="n">
-        <v>27.33504</v>
+        <v>48.3552</v>
       </c>
       <c r="J2" t="n">
-        <v>56.173</v>
+        <v>13.1236</v>
       </c>
       <c r="K2" t="n">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>custos_rs</t>
+          <t>planilha_custo</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>3%</t>
+          <t>planilha_ribbon</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -569,22 +569,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>3559</t>
+          <t>3562</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>30/06/2026 15:27:27</t>
+          <t>03/07/2026 09:26:03</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CITOPHARMA MANIPULAÇÃO DE MEDICAMENTOS ESPECIAIS LTDA</t>
+          <t>SAN GROUP BIOTECH BRASIL LTDA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>RIBBON CERA ARMOR 110x450 AWR1</t>
+          <t>RIBBON MISTO TRX45 110X450</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -593,31 +593,31 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>378.84</v>
+        <v>1348.56</v>
       </c>
       <c r="G3" t="n">
-        <v>221.88</v>
+        <v>806.4000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>11.3652</v>
+        <v>57.74</v>
       </c>
       <c r="I3" t="n">
-        <v>34.85328</v>
+        <v>124.06752</v>
       </c>
       <c r="J3" t="n">
-        <v>49.9105</v>
+        <v>44.6866</v>
       </c>
       <c r="K3" t="n">
-        <v>67</v>
+        <v>45</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>custos_rs</t>
+          <t>planilha_custo</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>3%</t>
+          <t>planilha_ribbon</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -632,22 +632,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3560</t>
+          <t>3563</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>30/06/2026 15:49:20</t>
+          <t>03/07/2026 15:32:12</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Gelico Gelatinas Indústria &amp; Comércio Ltda.</t>
+          <t>LONAX INDUSTRIA BRASILEIRA DE LONAS LTDA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ETIQUETA COUCHE BORRACHA ADESIVO HOTMELT 100X100 MM (500 UND X RL)</t>
+          <t>ETIQUETA ADESIVA SPOT 13MM AZUL 10000UN</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -656,18 +656,18 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>876.6</v>
+        <v>370</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>26.298</v>
+        <v>11.1</v>
       </c>
       <c r="I4" t="n">
-        <v>80.6472</v>
+        <v>34.04</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>qtd_rolo;tubete</t>
+          <t>dimensao;qtd_rolo;material;tubete</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -691,17 +691,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3561</t>
+          <t>3564</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>01/07/2026 13:28:50</t>
+          <t>06/07/2026 10:32:02</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>FRIGOBET FRIGORIFICO INDUSTRIAL BETIM LTDA</t>
+          <t>BMB - Belgo Mineira Bekaert Artefatos de Arame LTDA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -715,22 +715,22 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>525.6</v>
+        <v>645.36</v>
       </c>
       <c r="G5" t="n">
-        <v>360</v>
+        <v>343.2</v>
       </c>
       <c r="H5" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>48.3552</v>
+        <v>59.37312</v>
       </c>
       <c r="J5" t="n">
-        <v>13.1236</v>
+        <v>70.74209999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -754,144 +754,114 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3562</t>
+          <t>3565</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03/07/2026 09:26:03</t>
+          <t>06/07/2026 13:20:51</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SAN GROUP BIOTECH BRASIL LTDA</t>
+          <t>LONAX INDUSTRIA BRASILEIRA DE LONAS LTDA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>RIBBON MISTO TRX45 110X450</t>
+          <t>ETIQUETA ADESIVA SPOT 13MM AZUL 5000UN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Ribbon</t>
+          <t>Etiqueta Branca</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1348.56</v>
-      </c>
-      <c r="G6" t="n">
-        <v>806.4000000000001</v>
-      </c>
+        <v>370</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>57.74</v>
+        <v>11.1</v>
       </c>
       <c r="I6" t="n">
-        <v>124.06752</v>
-      </c>
-      <c r="J6" t="n">
-        <v>44.6866</v>
-      </c>
+        <v>34.04</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="n">
-        <v>45</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>planilha_custo</t>
-        </is>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>planilha_ribbon</t>
+          <t>3%</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr"/>
+          <t>custo incompleto</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>dimensao;qtd_rolo;material;tubete</t>
+        </is>
+      </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3563</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>03/07/2026 15:32:12</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>LONAX INDUSTRIA BRASILEIRA DE LONAS LTDA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>ETIQUETA ADESIVA SPOT 13MM AZUL 10000UN</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Etiqueta Branca</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>370</v>
-      </c>
+          <t>3566</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="I7" t="n">
-        <v>34.04</v>
-      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>3%</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>custo incompleto</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>dimensao;qtd_rolo;material;tubete</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>CANCELADA</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>NF cancelada</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3564</t>
+          <t>3567</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06/07/2026 10:32:02</t>
+          <t>06/07/2026 16:28:29</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BMB - Belgo Mineira Bekaert Artefatos de Arame LTDA</t>
+          <t>Fundação Filantrópica e Beneficiente de Saúde Arnaldo Gavazz</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>RIBBON CERA 110X450 EXTERNO</t>
+          <t>RIBBON CERA 110x65 EXTERNO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -900,22 +870,22 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>645.36</v>
+        <v>490.8</v>
       </c>
       <c r="G8" t="n">
-        <v>343.2</v>
+        <v>277.2</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>101.61</v>
       </c>
       <c r="I8" t="n">
-        <v>59.37312</v>
+        <v>45.1536</v>
       </c>
       <c r="J8" t="n">
-        <v>70.74209999999999</v>
+        <v>24.1113</v>
       </c>
       <c r="K8" t="n">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -939,114 +909,148 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3565</t>
+          <t>3567</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06/07/2026 13:20:51</t>
+          <t>06/07/2026 16:28:29</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LONAX INDUSTRIA BRASILEIRA DE LONAS LTDA</t>
+          <t>Fundação Filantrópica e Beneficiente de Saúde Arnaldo Gavazz</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ETIQUETA ADESIVA SPOT 13MM AZUL 5000UN</t>
+          <t>RIBBON MISTO TRX45 110X74</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Etiqueta Branca</t>
+          <t>Ribbon</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>370</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
+        <v>516.96</v>
+      </c>
+      <c r="G9" t="n">
+        <v>326.4</v>
+      </c>
       <c r="H9" t="n">
-        <v>11.1</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>34.04</v>
-      </c>
-      <c r="J9" t="inlineStr"/>
+        <v>47.56032</v>
+      </c>
+      <c r="J9" t="n">
+        <v>43.8112</v>
+      </c>
       <c r="K9" t="n">
-        <v>55</v>
-      </c>
-      <c r="L9" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>planilha_custo</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>3%</t>
+          <t>planilha_ribbon</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>custo incompleto</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>dimensao;qtd_rolo;material;tubete</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3566</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
+          <t>3568</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07/07/2026 15:33:36</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>San Group Biotech Brasil Ltda</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>RIBBON SUPER RESINA 110x74 EXTERNO - R400</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Ribbon</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>560.8</v>
+      </c>
+      <c r="G10" t="n">
+        <v>332</v>
+      </c>
+      <c r="H10" t="n">
+        <v>25</v>
+      </c>
+      <c r="I10" t="n">
+        <v>51.5936</v>
+      </c>
+      <c r="J10" t="n">
+        <v>45.8453</v>
+      </c>
       <c r="K10" t="n">
-        <v>48</v>
-      </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
+        <v>46</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>planilha_custo</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>planilha_ribbon</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>CANCELADA</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>NF cancelada</t>
-        </is>
-      </c>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3567</t>
+          <t>3569</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06/07/2026 16:28:29</t>
+          <t>08/07/2026 11:43:01</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fundação Filantrópica e Beneficiente de Saúde Arnaldo Gavazz</t>
+          <t>Fundação Dr. Amaral Carvalho</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RIBBON CERA 110x65 EXTERNO</t>
+          <t>RIBBON CERA 110X360 INTERNO - TDW108</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1055,22 +1059,22 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>490.8</v>
+        <v>1188</v>
       </c>
       <c r="G11" t="n">
-        <v>277.2</v>
+        <v>547.6800000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>101.61</v>
+        <v>153.14</v>
       </c>
       <c r="I11" t="n">
-        <v>45.1536</v>
+        <v>109.296</v>
       </c>
       <c r="J11" t="n">
-        <v>24.1113</v>
+        <v>68.99720000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -1094,22 +1098,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3567</t>
+          <t>3570</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06/07/2026 16:28:29</t>
+          <t>08/07/2026 13:29:47</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fundação Filantrópica e Beneficiente de Saúde Arnaldo Gavazz</t>
+          <t>ARGENTUM JOIAS LTDA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>RIBBON MISTO TRX45 110X74</t>
+          <t>RIBBON RESINA 110X74 EXTERNO - R200</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1118,22 +1122,22 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>516.96</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>326.4</v>
+        <v>18.58</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I12" t="n">
-        <v>47.56032</v>
+        <v>6.863199999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>43.8112</v>
+        <v>130.0151</v>
       </c>
       <c r="K12" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -1157,189 +1161,177 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3568</t>
+          <t>3571</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>07/07/2026 15:33:36</t>
+          <t>09/07/2026 09:28:28</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>San Group Biotech Brasil Ltda</t>
+          <t>FABRINIO SAMORA FERREIRA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>RIBBON SUPER RESINA 110x74 EXTERNO - R400</t>
+          <t>Faca Maciça 80x185x2 (MLC) para BOPP FASSON C2075</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ribbon</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>560.8</v>
-      </c>
-      <c r="G13" t="n">
-        <v>332</v>
-      </c>
+        <v>1042.02</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>25</v>
+        <v>31.2606</v>
       </c>
       <c r="I13" t="n">
-        <v>51.5936</v>
-      </c>
-      <c r="J13" t="n">
-        <v>45.8453</v>
-      </c>
+        <v>95.86583999999999</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>46</v>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>planilha_custo</t>
-        </is>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>planilha_ribbon</t>
+          <t>3%</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr"/>
+          <t>custo incompleto</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>segmento_sem_regra</t>
+        </is>
+      </c>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3569</t>
+          <t>3571</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>08/07/2026 11:43:01</t>
+          <t>09/07/2026 09:28:28</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fundação Dr. Amaral Carvalho</t>
+          <t>FABRINIO SAMORA FERREIRA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>RIBBON CERA 110X360 INTERNO - TDW108</t>
+          <t>Faca Maciça 50x30x1 (METALFLEXO) para BOPP FASSON S0290 - Maqflex</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Ribbon</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1188</v>
-      </c>
-      <c r="G14" t="n">
-        <v>547.6800000000001</v>
-      </c>
+        <v>895.47</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>153.14</v>
+        <v>26.8641</v>
       </c>
       <c r="I14" t="n">
-        <v>109.296</v>
-      </c>
-      <c r="J14" t="n">
-        <v>68.99720000000001</v>
-      </c>
+        <v>82.38324</v>
+      </c>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="n">
-        <v>62</v>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>planilha_custo</t>
-        </is>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>planilha_ribbon</t>
+          <t>3%</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr"/>
+          <t>custo incompleto</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>segmento_sem_regra</t>
+        </is>
+      </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>3570</t>
+          <t>3571</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>08/07/2026 13:29:47</t>
+          <t>09/07/2026 09:28:28</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ARGENTUM JOIAS LTDA</t>
+          <t>FABRINIO SAMORA FERREIRA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>RIBBON RESINA 110X74 EXTERNO - R200</t>
+          <t>Faca Maciça 100x80x2 (LEOFACAS) para Couchê Fasson Ecoprint S2045</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Ribbon</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>74.59999999999999</v>
-      </c>
-      <c r="G15" t="n">
-        <v>18.58</v>
-      </c>
+        <v>1000.42</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>25</v>
+        <v>30.0126</v>
       </c>
       <c r="I15" t="n">
-        <v>6.863199999999999</v>
-      </c>
-      <c r="J15" t="n">
-        <v>130.0151</v>
-      </c>
+        <v>92.03864</v>
+      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="n">
-        <v>30</v>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>planilha_custo</t>
-        </is>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>planilha_ribbon</t>
+          <t>3%</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr"/>
+          <t>custo incompleto</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>segmento_sem_regra</t>
+        </is>
+      </c>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
     </row>
@@ -1361,7 +1353,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Faca Maciça 80x185x2 (MLC) para BOPP FASSON C2075</t>
+          <t>Faca Maciça 102x197x2 (meio corte em 45mm)Fasson PP Branco Fosco NTC/C2075/60g</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1370,14 +1362,14 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1042.02</v>
+        <v>1045.88</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>31.2606</v>
+        <v>31.3764</v>
       </c>
       <c r="I16" t="n">
-        <v>95.86583999999999</v>
+        <v>96.22096000000001</v>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="n">
@@ -1405,103 +1397,115 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3571</t>
+          <t>3572</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>09/07/2026 09:28:28</t>
+          <t>09/07/2026 10:36:49</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>FABRINIO SAMORA FERREIRA</t>
+          <t>Nutrisantos Alimentação Animal LTDA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Faca Maciça 50x30x1 (METALFLEXO) para BOPP FASSON S0290 - Maqflex</t>
+          <t>ETIQUETA BOPP 100X50 ROLO COM 1500 TUBETE 3"</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Etiqueta Branca</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>895.47</v>
-      </c>
-      <c r="G17" t="inlineStr"/>
+        <v>3486.7</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2795.770599999999</v>
+      </c>
       <c r="H17" t="n">
-        <v>26.8641</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>82.38324</v>
-      </c>
-      <c r="J17" t="inlineStr"/>
+        <v>320.7764</v>
+      </c>
+      <c r="J17" t="n">
+        <v>13.2397</v>
+      </c>
       <c r="K17" t="n">
-        <v>31</v>
-      </c>
-      <c r="L17" t="inlineStr"/>
+        <v>41</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>planilha_jul26</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>3%</t>
+          <t>planilha_etiqueta</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>custo incompleto</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>segmento_sem_regra</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3571</t>
+          <t>3573</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>09/07/2026 09:28:28</t>
+          <t>10/07/2026 11:51:03</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>FABRINIO SAMORA FERREIRA</t>
+          <t>SUPREMO CARNES LTDA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Faca Maciça 100x80x2 (LEOFACAS) para Couchê Fasson Ecoprint S2045</t>
+          <t>RIBBON MISTO TRX45 83x450 EXTERNO</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Ribbon</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1000.42</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
+        <v>718.5599999999999</v>
+      </c>
+      <c r="G18" t="n">
+        <v>475.2</v>
+      </c>
       <c r="H18" t="n">
-        <v>30.0126</v>
+        <v>21.5568</v>
       </c>
       <c r="I18" t="n">
-        <v>92.03864</v>
-      </c>
-      <c r="J18" t="inlineStr"/>
+        <v>66.10751999999999</v>
+      </c>
+      <c r="J18" t="n">
+        <v>32.7642</v>
+      </c>
       <c r="K18" t="n">
-        <v>31</v>
-      </c>
-      <c r="L18" t="inlineStr"/>
+        <v>47</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>custos_rs</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr">
         <is>
           <t>3%</t>
@@ -1509,128 +1513,128 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>custo incompleto</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>segmento_sem_regra</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3571</t>
+          <t>3574</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>09/07/2026 09:28:28</t>
+          <t>13/07/2026 10:29:56</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>FABRINIO SAMORA FERREIRA</t>
+          <t>FRIGOBET FRIGORIFICO INDUSTRIAL BETIM LTDA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Faca Maciça 102x197x2 (meio corte em 45mm)Fasson PP Branco Fosco NTC/C2075/60g</t>
+          <t>RIBBON CERA 110X450 EXTERNO</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Ribbon</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1045.88</v>
-      </c>
-      <c r="G19" t="inlineStr"/>
+        <v>2102.4</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1440</v>
+      </c>
       <c r="H19" t="n">
-        <v>31.3764</v>
+        <v>120</v>
       </c>
       <c r="I19" t="n">
-        <v>96.22096000000001</v>
-      </c>
-      <c r="J19" t="inlineStr"/>
+        <v>193.4208</v>
+      </c>
+      <c r="J19" t="n">
+        <v>24.2347</v>
+      </c>
       <c r="K19" t="n">
-        <v>31</v>
-      </c>
-      <c r="L19" t="inlineStr"/>
+        <v>44</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>planilha_custo</t>
+        </is>
+      </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>3%</t>
+          <t>planilha_ribbon</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>custo incompleto</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>segmento_sem_regra</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>3572</t>
+          <t>3575</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>09/07/2026 10:36:49</t>
+          <t>13/07/2026 15:26:27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Nutrisantos Alimentação Animal LTDA</t>
+          <t>SUPREMO CARNES LTDA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ETIQUETA BOPP 100X50 ROLO COM 1500 TUBETE 3"</t>
+          <t>RIBBON MISTO TRX45 83x450 EXTERNO</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Etiqueta Branca</t>
+          <t>Ribbon</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>3486.7</v>
+        <v>718.5599999999999</v>
       </c>
       <c r="G20" t="n">
-        <v>2795.770599999999</v>
+        <v>475.2</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="I20" t="n">
-        <v>320.7764</v>
+        <v>66.10751999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>13.2397</v>
+        <v>24.6743</v>
       </c>
       <c r="K20" t="n">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>planilha_jul26</t>
+          <t>planilha_custo</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>planilha_etiqueta</t>
+          <t>planilha_ribbon</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1645,109 +1649,79 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3573</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>10/07/2026 11:51:03</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>SUPREMO CARNES LTDA</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>RIBBON MISTO TRX45 83x450 EXTERNO</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Ribbon</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>718.5599999999999</v>
-      </c>
-      <c r="G21" t="n">
-        <v>475.2</v>
-      </c>
-      <c r="H21" t="n">
-        <v>21.5568</v>
-      </c>
-      <c r="I21" t="n">
-        <v>66.10751999999999</v>
-      </c>
-      <c r="J21" t="n">
-        <v>32.7642</v>
-      </c>
+          <t>3576</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
-        <v>47</v>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>custos_rs</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>3%</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>AUSENTE</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Não existe no faturamento</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3574</t>
+          <t>3577</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>13/07/2026 10:29:56</t>
+          <t>14/07/2026 08:16:52</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FRIGOBET FRIGORIFICO INDUSTRIAL BETIM LTDA</t>
+          <t>ORGANIZACOES FRANCAP S/A</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>RIBBON CERA 110X450 EXTERNO</t>
+          <t>Etiqueta BOPP Fosco C2075 80x125 (rolo com 1.000) + Ribbon Misto 83x450</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Ribbon</t>
+          <t>Etiqueta Branca</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2102.4</v>
+        <v>19820</v>
       </c>
       <c r="G22" t="n">
-        <v>1440</v>
+        <v>12595</v>
       </c>
       <c r="H22" t="n">
-        <v>120</v>
+        <v>190</v>
       </c>
       <c r="I22" t="n">
-        <v>193.4208</v>
+        <v>1823.44</v>
       </c>
       <c r="J22" t="n">
-        <v>24.2347</v>
+        <v>41.378</v>
       </c>
       <c r="K22" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -1771,12 +1745,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3575</t>
+          <t>3578</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>13/07/2026 15:26:27</t>
+          <t>15/07/2026 08:23:51</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1795,22 +1769,22 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>718.5599999999999</v>
+        <v>2874.24</v>
       </c>
       <c r="G23" t="n">
-        <v>475.2</v>
+        <v>1900.8</v>
       </c>
       <c r="H23" t="n">
         <v>60</v>
       </c>
       <c r="I23" t="n">
-        <v>66.10751999999999</v>
+        <v>264.43008</v>
       </c>
       <c r="J23" t="n">
-        <v>24.6743</v>
+        <v>34.144</v>
       </c>
       <c r="K23" t="n">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -1834,88 +1808,118 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3576</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
+          <t>3579</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>15/07/2026 11:20:33</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Trindade Barbosa Análises Clínicas LTDA</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ETIQUETA BOPP 50X30 ROLO COM 1200</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Etiqueta Branca</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>2542.8</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1394.60192</v>
+      </c>
+      <c r="H24" t="n">
+        <v>15</v>
+      </c>
+      <c r="I24" t="n">
+        <v>233.9376</v>
+      </c>
+      <c r="J24" t="n">
+        <v>64.4815</v>
+      </c>
       <c r="K24" t="n">
-        <v>48</v>
-      </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
+        <v>50</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>planilha_jul26</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>planilha_etiqueta</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>AUSENTE</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>Não existe no faturamento</t>
-        </is>
-      </c>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>3577</t>
+          <t>3579</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>14/07/2026 08:16:52</t>
+          <t>15/07/2026 11:20:33</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ORGANIZACOES FRANCAP S/A</t>
+          <t>Trindade Barbosa Análises Clínicas LTDA</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Etiqueta BOPP Fosco C2075 80x125 (rolo com 1.000) + Ribbon Misto 83x450</t>
+          <t>ETIQUETA BOPP LATERAL LARANJA 50X30 ROLO COM 1200</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Etiqueta Branca</t>
+          <t>Etiqueta Colorida</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>19820</v>
+        <v>293.4</v>
       </c>
       <c r="G25" t="n">
-        <v>12595</v>
+        <v>163.13676</v>
       </c>
       <c r="H25" t="n">
-        <v>190</v>
+        <v>10</v>
       </c>
       <c r="I25" t="n">
-        <v>1823.44</v>
+        <v>26.9928</v>
       </c>
       <c r="J25" t="n">
-        <v>41.378</v>
+        <v>57.1732</v>
       </c>
       <c r="K25" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>planilha_custo</t>
+          <t>planilha_jul26</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>planilha_ribbon</t>
+          <t>planilha_etiqueta</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -1930,22 +1934,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>3578</t>
+          <t>3579</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>15/07/2026 08:23:51</t>
+          <t>15/07/2026 11:20:33</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SUPREMO CARNES LTDA</t>
+          <t>Trindade Barbosa Análises Clínicas LTDA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>RIBBON MISTO TRX45 83x450 EXTERNO</t>
+          <t>RIBBON MISTO TRX45 64x74 EXTERNO</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1954,22 +1958,22 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2874.24</v>
+        <v>538.3</v>
       </c>
       <c r="G26" t="n">
-        <v>1900.8</v>
+        <v>312.2</v>
       </c>
       <c r="H26" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="I26" t="n">
-        <v>264.43008</v>
+        <v>49.52359999999999</v>
       </c>
       <c r="J26" t="n">
-        <v>34.144</v>
+        <v>51.7541</v>
       </c>
       <c r="K26" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -1993,55 +1997,55 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3579</t>
+          <t>3580</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>15/07/2026 11:20:33</t>
+          <t>16/07/2026 09:50:49</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Trindade Barbosa Análises Clínicas LTDA</t>
+          <t>Indústria e Comércio Gomes Nogueira LTDA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>ETIQUETA BOPP 50X30 ROLO COM 1200</t>
+          <t>RIBBON CERA 110X74 EXTERNO</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Etiqueta Branca</t>
+          <t>Ribbon</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2542.8</v>
+        <v>292.8</v>
       </c>
       <c r="G27" t="n">
-        <v>1394.60192</v>
+        <v>127.68</v>
       </c>
       <c r="H27" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>233.9376</v>
+        <v>26.9376</v>
       </c>
       <c r="J27" t="n">
-        <v>64.4815</v>
+        <v>108.2256</v>
       </c>
       <c r="K27" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>planilha_jul26</t>
+          <t>planilha_custo</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>planilha_etiqueta</t>
+          <t>planilha_ribbon</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2056,55 +2060,55 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>3579</t>
+          <t>3581</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>15/07/2026 11:20:33</t>
+          <t>16/07/2026 15:11:03</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Trindade Barbosa Análises Clínicas LTDA</t>
+          <t>ONCOCLINICAS RIO DE JANEIRO S. A.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>ETIQUETA BOPP LATERAL LARANJA 50X30 ROLO COM 1200</t>
+          <t>RIBBON CERA 110X74 EXTERNO</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Etiqueta Colorida</t>
+          <t>Ribbon</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>293.4</v>
+        <v>376</v>
       </c>
       <c r="G28" t="n">
-        <v>163.13676</v>
+        <v>133</v>
       </c>
       <c r="H28" t="n">
-        <v>10</v>
+        <v>59</v>
       </c>
       <c r="I28" t="n">
-        <v>26.9928</v>
+        <v>34.592</v>
       </c>
       <c r="J28" t="n">
-        <v>57.1732</v>
+        <v>112.3368</v>
       </c>
       <c r="K28" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>planilha_jul26</t>
+          <t>planilha_custo</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>planilha_etiqueta</t>
+          <t>planilha_ribbon</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2119,22 +2123,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>3579</t>
+          <t>3582</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>15/07/2026 11:20:33</t>
+          <t>16/07/2026 15:44:08</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Trindade Barbosa Análises Clínicas LTDA</t>
+          <t>Hospital São Lucas de Governador Valadares Ltda</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>RIBBON MISTO TRX45 64x74 EXTERNO</t>
+          <t>RIBBON CERA 110X74 EXTERNO</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2143,22 +2147,22 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>538.3</v>
+        <v>460</v>
       </c>
       <c r="G29" t="n">
-        <v>312.2</v>
+        <v>266</v>
       </c>
       <c r="H29" t="n">
-        <v>15</v>
+        <v>47.81</v>
       </c>
       <c r="I29" t="n">
-        <v>49.52359999999999</v>
+        <v>42.32</v>
       </c>
       <c r="J29" t="n">
-        <v>51.7541</v>
+        <v>39.0489</v>
       </c>
       <c r="K29" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -2182,55 +2186,55 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3580</t>
+          <t>3583</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>16/07/2026 09:50:49</t>
+          <t>16/07/2026 17:37:22</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Indústria e Comércio Gomes Nogueira LTDA</t>
+          <t>Irmandade Nossa Senhora das Dores</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>RIBBON CERA 110X74 EXTERNO</t>
+          <t>ETIQUETA COUCHE 100X75 ROLO COM 358 TUBETE 1"</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Ribbon</t>
+          <t>Etiqueta Branca</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>292.8</v>
+        <v>2427</v>
       </c>
       <c r="G30" t="n">
-        <v>127.68</v>
+        <v>1573.38165</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>26.9376</v>
+        <v>223.284</v>
       </c>
       <c r="J30" t="n">
-        <v>108.2256</v>
+        <v>40.0624</v>
       </c>
       <c r="K30" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>planilha_custo</t>
+          <t>planilha_jul26</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>planilha_ribbon</t>
+          <t>planilha_etiqueta</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2245,22 +2249,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>3581</t>
+          <t>3583</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>16/07/2026 15:11:03</t>
+          <t>16/07/2026 17:37:22</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ONCOCLINICAS RIO DE JANEIRO S. A.</t>
+          <t>Irmandade Nossa Senhora das Dores</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>RIBBON CERA 110X74 EXTERNO</t>
+          <t>RIBBON MISTO TRX45 110X74</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2269,22 +2273,22 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>376</v>
+        <v>889</v>
       </c>
       <c r="G31" t="n">
-        <v>133</v>
+        <v>680</v>
       </c>
       <c r="H31" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>34.592</v>
+        <v>81.788</v>
       </c>
       <c r="J31" t="n">
-        <v>112.3368</v>
+        <v>18.7076</v>
       </c>
       <c r="K31" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -2308,22 +2312,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>3582</t>
+          <t>3584</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>16/07/2026 15:44:08</t>
+          <t>20/07/2026 08:40:09</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Hospital São Lucas de Governador Valadares Ltda</t>
+          <t>CIA DE FIACAO E TECIDOS CEDRO E CACHOEIRA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>RIBBON CERA 110X74 EXTERNO</t>
+          <t>RIBBON CERA 110x360 INTERNO</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2332,26 +2336,26 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>460</v>
+        <v>556</v>
       </c>
       <c r="G32" t="n">
-        <v>266</v>
+        <v>228.2</v>
       </c>
       <c r="H32" t="n">
-        <v>47.81</v>
+        <v>40</v>
       </c>
       <c r="I32" t="n">
-        <v>42.32</v>
+        <v>51.152</v>
       </c>
       <c r="J32" t="n">
-        <v>39.0489</v>
+        <v>103.702</v>
       </c>
       <c r="K32" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>planilha_custo</t>
+          <t>planilha_ribbon</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2371,55 +2375,55 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>3583</t>
+          <t>3585</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>16/07/2026 17:37:22</t>
+          <t>20/07/2026 09:45:59</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Irmandade Nossa Senhora das Dores</t>
+          <t>Musashi do Brasil LTDA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ETIQUETA COUCHE 100X75 ROLO COM 358 TUBETE 1"</t>
+          <t>RIBBON SUPER RESINA 110x74 EXTERNO - R400</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Etiqueta Branca</t>
+          <t>Ribbon</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2427</v>
+        <v>1820</v>
       </c>
       <c r="G33" t="n">
-        <v>1573.38165</v>
+        <v>1162</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I33" t="n">
-        <v>223.284</v>
+        <v>167.44</v>
       </c>
       <c r="J33" t="n">
-        <v>40.0624</v>
+        <v>39.6351</v>
       </c>
       <c r="K33" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>planilha_jul26</t>
+          <t>planilha_custo</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>planilha_etiqueta</t>
+          <t>planilha_ribbon</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2434,22 +2438,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>3583</t>
+          <t>3586</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>16/07/2026 17:37:22</t>
+          <t>21/07/2026 11:32:16</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Irmandade Nossa Senhora das Dores</t>
+          <t>Centrasa - Centro de Serviços do Aço LTDA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>RIBBON MISTO TRX45 110X74</t>
+          <t>RIBBON CERA 110X300 EXTERNO</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2458,19 +2462,19 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>889</v>
+        <v>704.7</v>
       </c>
       <c r="G34" t="n">
-        <v>680</v>
+        <v>288.3</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I34" t="n">
-        <v>81.788</v>
+        <v>64.83240000000001</v>
       </c>
       <c r="J34" t="n">
-        <v>18.7076</v>
+        <v>104.602</v>
       </c>
       <c r="K34" t="n">
         <v>47</v>
@@ -2497,55 +2501,55 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>3584</t>
+          <t>3587</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>20/07/2026 08:40:09</t>
+          <t>22/07/2026 10:32:02</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CIA DE FIACAO E TECIDOS CEDRO E CACHOEIRA</t>
+          <t>Nutrisantos Alimentação Animal LTDA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>RIBBON CERA 110x360 INTERNO</t>
+          <t>ETIQUETA COUCHE 100X50 ROLO COM 1000 TUBETE 1"</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Ribbon</t>
+          <t>Etiqueta Branca</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>556</v>
+        <v>1277</v>
       </c>
       <c r="G35" t="n">
-        <v>228.2</v>
+        <v>998.3200000000002</v>
       </c>
       <c r="H35" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>51.152</v>
+        <v>117.484</v>
       </c>
       <c r="J35" t="n">
-        <v>103.702</v>
+        <v>16.1467</v>
       </c>
       <c r="K35" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>planilha_ribbon</t>
+          <t>planilha_jul26</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>planilha_ribbon</t>
+          <t>planilha_etiqueta</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2560,55 +2564,55 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>3585</t>
+          <t>3588</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>20/07/2026 09:45:59</t>
+          <t>22/07/2026 10:37:27</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Musashi do Brasil LTDA</t>
+          <t>Nutrisantos Alimentação Animal LTDA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>RIBBON SUPER RESINA 110x74 EXTERNO - R400</t>
+          <t>ETIQUETA BOPP 100X150 ROLO COM 1500 TUBETE 3"</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Ribbon</t>
+          <t>Etiqueta Branca</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>1820</v>
+        <v>8553</v>
       </c>
       <c r="G36" t="n">
-        <v>1162</v>
+        <v>6517.204799999999</v>
       </c>
       <c r="H36" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>167.44</v>
+        <v>786.876</v>
       </c>
       <c r="J36" t="n">
-        <v>39.6351</v>
+        <v>19.1634</v>
       </c>
       <c r="K36" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>planilha_custo</t>
+          <t>planilha_jul26</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>planilha_ribbon</t>
+          <t>planilha_etiqueta</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2623,22 +2627,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>3586</t>
+          <t>3588</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>21/07/2026 11:32:16</t>
+          <t>22/07/2026 10:37:27</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Centrasa - Centro de Serviços do Aço LTDA</t>
+          <t>Nutrisantos Alimentação Animal LTDA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>RIBBON CERA 110X300 EXTERNO</t>
+          <t>RIBBON MISTO TRX45 110X300</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2647,22 +2651,22 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>704.7</v>
+        <v>2037</v>
       </c>
       <c r="G37" t="n">
-        <v>288.3</v>
+        <v>1317.6</v>
       </c>
       <c r="H37" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>64.83240000000001</v>
+        <v>187.404</v>
       </c>
       <c r="J37" t="n">
-        <v>104.602</v>
+        <v>40.3761</v>
       </c>
       <c r="K37" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -2686,55 +2690,55 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>3587</t>
+          <t>3589</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>22/07/2026 10:32:02</t>
+          <t>23/07/2026 11:55:13</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Nutrisantos Alimentação Animal LTDA</t>
+          <t>SADA Transportes e Armazenagens LTDA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>ETIQUETA COUCHE 100X50 ROLO COM 1000 TUBETE 1"</t>
+          <t>RIBBON ZEBRA  800300-350/250BR PARA ZC300/ZC100</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Etiqueta Branca</t>
+          <t>Suprimentos</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>1277</v>
+        <v>928.36</v>
       </c>
       <c r="G38" t="n">
-        <v>998.3200000000002</v>
+        <v>534</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="I38" t="n">
-        <v>117.484</v>
+        <v>85.40912</v>
       </c>
       <c r="J38" t="n">
-        <v>16.1467</v>
+        <v>46.62</v>
       </c>
       <c r="K38" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>planilha_jul26</t>
+          <t>planilha_custo</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>planilha_etiqueta</t>
+          <t>planilha_ribbon</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2749,55 +2753,55 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>3588</t>
+          <t>3590</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>22/07/2026 10:37:27</t>
+          <t>23/07/2026 13:54:15</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Nutrisantos Alimentação Animal LTDA</t>
+          <t>FUNDACAO DOUTOR AMARAL CARVALHO</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>ETIQUETA BOPP 100X150 ROLO COM 1500 TUBETE 3"</t>
+          <t>RIBBON CERA 110X360 INTERNO - TDW108</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Etiqueta Branca</t>
+          <t>Ribbon</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>8553</v>
+        <v>1485</v>
       </c>
       <c r="G39" t="n">
-        <v>6517.204799999999</v>
+        <v>684.6</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>137.74</v>
       </c>
       <c r="I39" t="n">
-        <v>786.876</v>
+        <v>136.62</v>
       </c>
       <c r="J39" t="n">
-        <v>19.1634</v>
+        <v>76.839</v>
       </c>
       <c r="K39" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>planilha_jul26</t>
+          <t>planilha_custo</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>planilha_etiqueta</t>
+          <t>planilha_ribbon</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2812,22 +2816,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>3588</t>
+          <t>3591</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>22/07/2026 10:37:27</t>
+          <t>27/07/2026 10:51:57</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Nutrisantos Alimentação Animal LTDA</t>
+          <t>Indústria de Carnes Grandminas LTDA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>RIBBON MISTO TRX45 110X300</t>
+          <t>RIBBON CERA 110X450 EXTERNO</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2836,22 +2840,22 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>2037</v>
+        <v>1137.12</v>
       </c>
       <c r="G40" t="n">
-        <v>1317.6</v>
+        <v>686.4000000000001</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="I40" t="n">
-        <v>187.404</v>
+        <v>104.61504</v>
       </c>
       <c r="J40" t="n">
-        <v>40.3761</v>
+        <v>41.682</v>
       </c>
       <c r="K40" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -2875,55 +2879,55 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>3589</t>
+          <t>3592</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>23/07/2026 11:55:13</t>
+          <t>27/07/2026 13:18:12</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SADA Transportes e Armazenagens LTDA</t>
+          <t>LONAX INDUSTRIA BRASILEIRA DE LONAS LTDA</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>RIBBON ZEBRA  800300-350/250BR PARA ZC300/ZC100</t>
+          <t>ETIQUETA BOPP 100X100 (30M) TUBETE 1" - 1 COLUNA</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Suprimentos</t>
+          <t>Etiqueta Branca</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>928.36</v>
+        <v>1017.2</v>
       </c>
       <c r="G41" t="n">
-        <v>534</v>
+        <v>578.5897281553398</v>
       </c>
       <c r="H41" t="n">
-        <v>60</v>
+        <v>59.34</v>
       </c>
       <c r="I41" t="n">
-        <v>85.40912</v>
+        <v>93.58240000000001</v>
       </c>
       <c r="J41" t="n">
-        <v>46.62</v>
+        <v>49.3766</v>
       </c>
       <c r="K41" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>planilha_custo</t>
+          <t>planilha_jul26</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>planilha_ribbon</t>
+          <t>planilha_etiqueta</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -2938,22 +2942,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>3590</t>
+          <t>3593</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>23/07/2026 13:54:15</t>
+          <t>27/07/2026 16:01:31</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>FUNDACAO DOUTOR AMARAL CARVALHO</t>
+          <t>PROFARMA DISTRIBUIDORA DE PRODUTOS FARMACEUTICOS SA - RS</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>RIBBON CERA 110X360 INTERNO - TDW108</t>
+          <t>RIBBON CERA 110X74 EXTERNO</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2962,22 +2966,22 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>1485</v>
+        <v>1673.28</v>
       </c>
       <c r="G42" t="n">
-        <v>684.6</v>
+        <v>760.3200000000001</v>
       </c>
       <c r="H42" t="n">
-        <v>137.74</v>
+        <v>300</v>
       </c>
       <c r="I42" t="n">
-        <v>136.62</v>
+        <v>153.94176</v>
       </c>
       <c r="J42" t="n">
-        <v>76.839</v>
+        <v>60.3717</v>
       </c>
       <c r="K42" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
@@ -3001,22 +3005,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>3591</t>
+          <t>3594</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>27/07/2026 10:51:57</t>
+          <t>29/07/2026 08:14:24</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Indústria de Carnes Grandminas LTDA</t>
+          <t>PROFARMA DISTRIBUIDORA DE PRODUTOS FARMACEUTICOS SA - RJ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>RIBBON CERA 110X450 EXTERNO</t>
+          <t>RIBBON CERA 110X74 EXTERNO</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3025,22 +3029,22 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>1137.12</v>
+        <v>1673.28</v>
       </c>
       <c r="G43" t="n">
-        <v>686.4000000000001</v>
+        <v>760.3200000000001</v>
       </c>
       <c r="H43" t="n">
-        <v>60</v>
+        <v>199.5</v>
       </c>
       <c r="I43" t="n">
-        <v>104.61504</v>
+        <v>153.94176</v>
       </c>
       <c r="J43" t="n">
-        <v>41.682</v>
+        <v>73.5898</v>
       </c>
       <c r="K43" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -3064,22 +3068,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>3592</t>
+          <t>3595</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>27/07/2026 13:18:12</t>
+          <t>29/07/2026 13:17:40</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>LONAX INDUSTRIA BRASILEIRA DE LONAS LTDA</t>
+          <t>Instituto de Previdência dos Servidores do Estado MG</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>ETIQUETA BOPP 100X100 (30M) TUBETE 1" - 1 COLUNA</t>
+          <t>ETIQUETA COUCHE 100X85 ROLO COM 500 TUBETE 1"</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3088,22 +3092,22 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>1017.2</v>
+        <v>492</v>
       </c>
       <c r="G44" t="n">
-        <v>578.5897281553398</v>
+        <v>326.8976</v>
       </c>
       <c r="H44" t="n">
-        <v>59.34</v>
+        <v>20</v>
       </c>
       <c r="I44" t="n">
-        <v>93.58240000000001</v>
+        <v>45.264</v>
       </c>
       <c r="J44" t="n">
-        <v>49.3766</v>
+        <v>30.5412</v>
       </c>
       <c r="K44" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
@@ -3127,55 +3131,55 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>3593</t>
+          <t>3595</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>27/07/2026 16:01:31</t>
+          <t>29/07/2026 13:17:40</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PROFARMA DISTRIBUIDORA DE PRODUTOS FARMACEUTICOS SA - RS</t>
+          <t>Instituto de Previdência dos Servidores do Estado MG</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>RIBBON CERA 110X74 EXTERNO</t>
+          <t>ETIQUETA COUCHE 48X33 ROLO COM 2500 TUBETE 1"</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Ribbon</t>
+          <t>Etiqueta Branca</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>1673.28</v>
+        <v>552.2</v>
       </c>
       <c r="G45" t="n">
-        <v>760.3200000000001</v>
+        <v>352.4439999999999</v>
       </c>
       <c r="H45" t="n">
-        <v>300</v>
+        <v>25</v>
       </c>
       <c r="I45" t="n">
-        <v>153.94176</v>
+        <v>50.80240000000001</v>
       </c>
       <c r="J45" t="n">
-        <v>60.3717</v>
+        <v>35.1697</v>
       </c>
       <c r="K45" t="n">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>planilha_custo</t>
+          <t>planilha_jul26</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>planilha_ribbon</t>
+          <t>planilha_etiqueta</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3190,22 +3194,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>3594</t>
+          <t>3596</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>29/07/2026 08:14:24</t>
+          <t>30/07/2026 14:58:06</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PROFARMA DISTRIBUIDORA DE PRODUTOS FARMACEUTICOS SA - RJ</t>
+          <t>BMB - Belgo Mineira Bekaert Artefatos de Arame LTDA</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>RIBBON CERA 110X74 EXTERNO</t>
+          <t>RIBBON CERA 110X450 EXTERNO</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -3214,22 +3218,22 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>1673.28</v>
+        <v>645.36</v>
       </c>
       <c r="G46" t="n">
-        <v>760.3200000000001</v>
+        <v>343.2</v>
       </c>
       <c r="H46" t="n">
-        <v>199.5</v>
+        <v>0</v>
       </c>
       <c r="I46" t="n">
-        <v>153.94176</v>
+        <v>59.37312</v>
       </c>
       <c r="J46" t="n">
-        <v>73.5898</v>
+        <v>70.74209999999999</v>
       </c>
       <c r="K46" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
@@ -3253,55 +3257,55 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>3595</t>
+          <t>3597</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>29/07/2026 13:17:40</t>
+          <t>30/07/2026 15:50:42</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Instituto de Previdência dos Servidores do Estado MG</t>
+          <t>FUNDACAO DOUTOR AMARAL CARVALHO</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ETIQUETA COUCHE 100X85 ROLO COM 500 TUBETE 1"</t>
+          <t>RIBBON CERA 110X360 INTERNO - TDW108</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Etiqueta Branca</t>
+          <t>Ribbon</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>492</v>
+        <v>1188</v>
       </c>
       <c r="G47" t="n">
-        <v>326.8976</v>
+        <v>547.6800000000001</v>
       </c>
       <c r="H47" t="n">
-        <v>20</v>
+        <v>219.41</v>
       </c>
       <c r="I47" t="n">
-        <v>45.264</v>
+        <v>109.296</v>
       </c>
       <c r="J47" t="n">
-        <v>30.5412</v>
+        <v>56.8971</v>
       </c>
       <c r="K47" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>planilha_jul26</t>
+          <t>planilha_custo</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>planilha_etiqueta</t>
+          <t>planilha_ribbon</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3316,55 +3320,55 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>3595</t>
+          <t>3597</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>29/07/2026 13:17:40</t>
+          <t>30/07/2026 15:50:42</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Instituto de Previdência dos Servidores do Estado MG</t>
+          <t>FUNDACAO DOUTOR AMARAL CARVALHO</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>ETIQUETA COUCHE 48X33 ROLO COM 2500 TUBETE 1"</t>
+          <t>RIBBON CERA 110x74 EXTERNO G42</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Etiqueta Branca</t>
+          <t>Ribbon</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>552.2</v>
+        <v>184.5</v>
       </c>
       <c r="G48" t="n">
-        <v>352.4439999999999</v>
+        <v>126.45</v>
       </c>
       <c r="H48" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I48" t="n">
-        <v>50.80240000000001</v>
+        <v>16.974</v>
       </c>
       <c r="J48" t="n">
-        <v>35.1697</v>
+        <v>32.484</v>
       </c>
       <c r="K48" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>planilha_jul26</t>
+          <t>planilha_ribbon</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>planilha_etiqueta</t>
+          <t>planilha_ribbon</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3379,17 +3383,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>3596</t>
+          <t>3598</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>30/07/2026 14:58:06</t>
+          <t>31/07/2026 10:00:53</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>BMB - Belgo Mineira Bekaert Artefatos de Arame LTDA</t>
+          <t>META INDUSTRIA DE CALCADOS LTDA</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3403,22 +3407,22 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>645.36</v>
+        <v>2352</v>
       </c>
       <c r="G49" t="n">
-        <v>343.2</v>
+        <v>1372.8</v>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="I49" t="n">
-        <v>59.37312</v>
+        <v>216.384</v>
       </c>
       <c r="J49" t="n">
-        <v>70.74209999999999</v>
+        <v>46.8252</v>
       </c>
       <c r="K49" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
@@ -3438,313 +3442,6 @@
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>3597</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>30/07/2026 15:50:42</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>FUNDACAO DOUTOR AMARAL CARVALHO</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>RIBBON CERA 110X360 INTERNO - TDW108</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Ribbon</t>
-        </is>
-      </c>
-      <c r="F50" t="n">
-        <v>1188</v>
-      </c>
-      <c r="G50" t="n">
-        <v>547.6800000000001</v>
-      </c>
-      <c r="H50" t="n">
-        <v>219.41</v>
-      </c>
-      <c r="I50" t="n">
-        <v>109.296</v>
-      </c>
-      <c r="J50" t="n">
-        <v>56.8971</v>
-      </c>
-      <c r="K50" t="n">
-        <v>45</v>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>planilha_custo</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>planilha_ribbon</t>
-        </is>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>3597</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>30/07/2026 15:50:42</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>FUNDACAO DOUTOR AMARAL CARVALHO</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>RIBBON CERA 110x74 EXTERNO G42</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Ribbon</t>
-        </is>
-      </c>
-      <c r="F51" t="n">
-        <v>184.5</v>
-      </c>
-      <c r="G51" t="n">
-        <v>126.45</v>
-      </c>
-      <c r="H51" t="n">
-        <v>0</v>
-      </c>
-      <c r="I51" t="n">
-        <v>16.974</v>
-      </c>
-      <c r="J51" t="n">
-        <v>32.484</v>
-      </c>
-      <c r="K51" t="n">
-        <v>45</v>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>planilha_ribbon</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>planilha_ribbon</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>3598</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>31/07/2026 10:00:53</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>META INDUSTRIA DE CALCADOS LTDA</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>RIBBON CERA 110X450 EXTERNO</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Ribbon</t>
-        </is>
-      </c>
-      <c r="F52" t="n">
-        <v>2352</v>
-      </c>
-      <c r="G52" t="n">
-        <v>1372.8</v>
-      </c>
-      <c r="H52" t="n">
-        <v>120</v>
-      </c>
-      <c r="I52" t="n">
-        <v>216.384</v>
-      </c>
-      <c r="J52" t="n">
-        <v>46.8252</v>
-      </c>
-      <c r="K52" t="n">
-        <v>47</v>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>planilha_custo</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>planilha_ribbon</t>
-        </is>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>1063</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>03/08/2022 11:00:00</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>ACG DO BRASIL S/A</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Bateria Lap Top Dell 3480 Modelo 33YDH</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Suprimentos</t>
-        </is>
-      </c>
-      <c r="F53" t="n">
-        <v>1224.58</v>
-      </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="n">
-        <v>36.73739999999999</v>
-      </c>
-      <c r="I53" t="n">
-        <v>112.66136</v>
-      </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>3%</t>
-        </is>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>custo incompleto</t>
-        </is>
-      </c>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t>custo_rs</t>
-        </is>
-      </c>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>1063</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>18/05/2026 14:15:48</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Scientific Dental Medical LTDA</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>ETIQUETA COUCHE 100X100 ROLO COM 400 TUBETE 1"</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Etiqueta Branca</t>
-        </is>
-      </c>
-      <c r="F54" t="n">
-        <v>4354</v>
-      </c>
-      <c r="G54" t="n">
-        <v>3002.2288</v>
-      </c>
-      <c r="H54" t="n">
-        <v>130.62</v>
-      </c>
-      <c r="I54" t="n">
-        <v>400.568</v>
-      </c>
-      <c r="J54" t="n">
-        <v>27.3325</v>
-      </c>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>rolo</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>3%</t>
-        </is>
-      </c>
-      <c r="N54" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>